<commit_message>
feat: implement R-45/R-49/R-50 (mute-by-default, realistic surface views, photo rename/delete)
- R-45: Game starts muted (🔇); first mute-btn click initializes audio and unmutes
- R-49: Rewrote drawSurfaceView() for Mercury/Venus/Earth/Mars/Saturn/Uranus with
  planet-specific sky colors, cloud layers, terrain features, and lighting
- R-50: Added ✏ rename and 🗑 delete buttons to photo cards; synced with IndexedDB

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PALE_BLUE_DOT_修正要望管理表.xlsx
+++ b/docs/PALE_BLUE_DOT_修正要望管理表.xlsx
@@ -1534,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1701,6 +1701,28 @@
       <c r="D8" s="21" t="inlineStr">
         <is>
           <t>R-37〜R-51のうち10件実装。地表ドラッグ/自転修正/ハードリロード/アイコン品質/サウンド制御/帰還演出リニューアル</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>更新</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>R-45/R-49/R-50 実装完了。全15件のうち計13件が完了（R-45:初期ミュート、R-49:地表描画リアル化6惑星、R-50:写真削除/名前変更機能）</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2908,7 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
@@ -3054,7 +3076,7 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
@@ -3096,7 +3118,7 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">

</xml_diff>

<commit_message>
docs: add 修正要望_v2.3 sheet (R-52~R-57) and update code conventions
- 修正要望管理表: 第3回テスト(2026-04-04)結果を反映した修正要望_v2.3シートを追加
  - R-52: TC17 アイコン半影問題（R-40未解決）
  - R-53: TC22 地表ドラッグ不可（R-37未解決 / surface-ui z-index遮断が原因）
  - R-54: TC21/TC62-67 地表描画リアル化（R-49対応済、再テスト要）
  - R-55: TC72 ダウンロードファイル名固定バグ
  - R-56: TC75 自転速度下限調整（R-38未解決）
  - R-57: 月の追加（改善要望書No.20）
- コード規約 v1.1: R-45/R-49/R-50反映、surface-uiドラッグ注意事項、
  地表ビュー描画規約セクション追加、simSpeed表記更新

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PALE_BLUE_DOT_修正要望管理表.xlsx
+++ b/docs/PALE_BLUE_DOT_修正要望管理表.xlsx
@@ -11,6 +11,7 @@
     <sheet name="修正履歴" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="修正要望_v2.1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="修正要望_v2.2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="修正要望_v2.3" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,8 +108,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="MS Gothic"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -195,8 +201,18 @@
         <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -218,11 +234,25 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -298,6 +328,27 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1534,7 +1585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1723,6 +1774,28 @@
       <c r="D9" s="21" t="inlineStr">
         <is>
           <t>R-45/R-49/R-50 実装完了。全15件のうち計13件が完了（R-45:初期ミュート、R-49:地表描画リアル化6惑星、R-50:写真削除/名前変更機能）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>追記</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>修正要望_v2.3シート追加（R-52〜R-57）。第3回テスト（2026-04-04）結果を反映。TC17/TC22/TC72/TC75の残存バグと、TC21/TC62〜TC67のR-49再テスト要確認、改善要望書No.20（月の追加）を新規起票</t>
         </is>
       </c>
     </row>
@@ -3180,4 +3253,343 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>PALE BLUE DOT  修正要望管理表  v2.2テスト後（Chrome PC  第3回テスト）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>管理No.</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>要望内容</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>関連TC</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>優先度</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>ステータス</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>対応方針（案）</t>
+        </is>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="65" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>R-52</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>改善要望（再修正）</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>情報パネルの惑星アイコンが常に半影になっている（R-40未解決）</t>
+        </is>
+      </c>
+      <c r="D3" s="29" t="inlineStr">
+        <is>
+          <t>TC17</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F3" s="30" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="G3" s="29" t="inlineStr">
+        <is>
+          <t>drawIconFrame()内のbrightness(1.6)フィルターでは元テクスチャに焼き込まれたLambertシェーディングのグラデーションを消せない。フィルターをbrightness(3) saturate(0.9) contrast(1.1)の複合指定に強化するか、ictxでdrawImage後にglobalCompositeOperation="screen"で白グラデーションをオーバーレイしシャドウ側を強制的に明るくする。</t>
+        </is>
+      </c>
+      <c r="H3" s="29" t="inlineStr">
+        <is>
+          <t>R-40で対応済とされていたが第3回テストでも△が継続。「常に半分影」の根本原因はCanvasテクスチャ生成時に焼き込まれた暗半球グラデーション。brightness(1.6)では消去不十分</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="65" customHeight="1">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>R-53</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>バグ（再修正）</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>地表ビューでマウスドラッグが効かない（R-37再修正）</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>TC22</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>surface-ui(z-index:56)がsurface-canvas(z-index:55)の全面を覆っており、surface-canvasへのmousedown/mousemoveイベントが届かない。修正方針：ドラッグリスナーをsurface-canvas→surface-uiに移動。ただしボタン要素(button)上でのmousedownはe.target.tagName==='BUTTON'で除外し、ドラッグ判定はsurface-ui全体で行う。</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>R-37でsurface-canvasにリスナーを追加したが、z-index上位のsurface-uiがイベントを遮断していたため×が継続。ボタン(「宇宙へ戻る」「嵐を止める」)は固有クリックハンドラを持つため影響なし</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="65" customHeight="1">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>R-54</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>確認（再テスト要）</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>地表ビュー描画リアル化（R-49対応済、再テスト要）</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>TC21 / TC62〜TC67</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>対応済</t>
+        </is>
+      </c>
+      <c r="G5" s="29" t="inlineStr">
+        <is>
+          <t>2026-04-05付けでR-49として6惑星（水星/金星/地球/火星/土星/天王星）のdrawSurfaceView()を全面書き直し済み。第3回テストはR-49実装前日（2026-04-04）に実施されたため△が残存。第4回テストで合否を確認。追加改善が必要な場合は新規Rとして起票。</t>
+        </is>
+      </c>
+      <c r="H5" s="29" t="inlineStr">
+        <is>
+          <t>TC21（地表ビュー表示）は備考なし△のためTC62〜TC67と同一原因（描画品質）と判断。R-49コミット: f41804d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>R-55</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>バグ</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>ダウンロード時のファイル名がアルバム内表示名と異なる</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>TC72</t>
+        </is>
+      </c>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="G6" s="31" t="inlineStr">
+        <is>
+          <t>photo-dl-btnのa.download属性が固定値'pale-blue-dot-photo.png'になっている。ph.labelを用いたファイル名生成に変更：
+a.download = (ph.label||'photo').replace(/[\/\?%*:|"&lt;&gt;]/g,'_') + '.png'
+R-50で実装した「名前変更」機能との連携も確認。名前変更後のラベルもダウンロード名に反映させる。</t>
+        </is>
+      </c>
+      <c r="H6" s="31" t="inlineStr">
+        <is>
+          <t>R-50（名前変更/削除）では対応済みだがダウンロードファイル名は別件として残存。対応工数は軽微（1行修正）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="65" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>R-56</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>バグ（再修正）</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>惑星自転速度がsimSpeed変化に連動せずわかりづらい（R-38再修正）</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>TC75</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>R-38でMath.max(1, simSpeed)を採用した結果、simSpeed=0〜1の全域で自転速度が1×固定になり変化が視認できない。
+修正方針：Math.max(0.5, simSpeed)に変更。
+・simSpeed &lt; 0.5 → 自転速度 = rotSpeed * dt * 0.5（下限固定）
+・simSpeed &gt;= 0.5 → 自転速度 = rotSpeed * dt * simSpeed（線形スケール）
+公転計算はsimSpeedを直接使用するため変更不要。</t>
+        </is>
+      </c>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>R-38で「Math.max(1,s)」を採用したがsimSpeed=1では変化が見えず×が継続。ユーザー仕様：「時間速度0.5時と同様の速度を下限にし、以下には下げない。公転速度のみ下げる」</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="65" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>R-57</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>新機能</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>月の追加（地球周回・公転・自転・情報パネル）</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>新規（改善要望書No.20）</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>改善要望書No.20に対応。実装方針：
+① buildMoon()：SphereGeometry + CanvasTexture（灰色、クレーター模様）でMesh生成
+② 地球のchildren配列に追加し地球基準の相対位置で公転軌道を設定
+③ 自転・公転アニメーションをanimateループに追加（他惑星と同様のrotSpeed/orbitRadiusプロパティ）
+④ クリック時の情報パネル対応（質量：7.35×10²²kg、半径：1737km、平均距離：38.4万km）
+⑤ コレクションスロット追加の要否を別途確認</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>改善要望書No.20：「地球の周りに月を配置。地球の周りを公転しながら自転する様子を地球などの惑星と同様に表現。公転運動及び自転運動や情報パネルに関する設定も、ほかの惑星とすべて同様とする。」</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>